<commit_message>
fix: keep an external hyperlink's relationship ID on save (#705)
A hyperlink now keeps the relationship ID it was loaded with, while its
address is unchanged and no other relationship in the sheet's part uses
the ID. The generator reserves the kept ID so no later part in the save
takes it. A copied hyperlink or one whose address changes gets a new ID.

A sheet with an external hyperlink now saves the same bytes when loaded
and saved, so #702 can leave its part as the file had it. The
Hyperlinks example reference file keeps rId6-rId10 instead of being
renumbered to rId13-rId17.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/Misc/Hyperlinks.xlsx
+++ b/XLibur.Tests/Resource/Examples/Misc/Hyperlinks.xlsx
@@ -509,15 +509,15 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink ref="A1" r:id="rId13"/>
-    <x:hyperlink ref="A2" r:id="rId14" tooltip="Click to go to Yahoo!"/>
+    <x:hyperlink ref="A1" r:id="rId6"/>
+    <x:hyperlink ref="A2" r:id="rId7" tooltip="Click to go to Yahoo!"/>
     <x:hyperlink ref="A3" location="Hyperlinks!Test.xlsx" display="Link to a file - same folder"/>
-    <x:hyperlink ref="A4" r:id="rId15"/>
-    <x:hyperlink ref="A5" r:id="rId16"/>
+    <x:hyperlink ref="A4" r:id="rId8"/>
+    <x:hyperlink ref="A5" r:id="rId9"/>
     <x:hyperlink ref="A6" location="Hyperlinks!B1" display="Link to an address in this worksheet"/>
     <x:hyperlink ref="A7" location="'Second Sheet'!A1" display="Link to an address in another worksheet"/>
     <x:hyperlink ref="A8" location="Hyperlinks!B1:C2" tooltip="SquareBox" display="Link to a range in this worksheet"/>
-    <x:hyperlink ref="A9" r:id="rId17"/>
+    <x:hyperlink ref="A9" r:id="rId10"/>
     <x:hyperlink ref="A11" location="Hyperlinks!B1:C2" display="Odd looking link"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
fix: keep an external hyperlink's relationship ID on save (#705) (#710)
A hyperlink now keeps the relationship ID it was loaded with, while its
address is unchanged and no other relationship in the sheet's part uses
the ID. The generator reserves the kept ID so no later part in the save
takes it. A copied hyperlink or one whose address changes gets a new ID.

A sheet with an external hyperlink now saves the same bytes when loaded
and saved, so #702 can leave its part as the file had it. The
Hyperlinks example reference file keeps rId6-rId10 instead of being
renumbered to rId13-rId17.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/Misc/Hyperlinks.xlsx
+++ b/XLibur.Tests/Resource/Examples/Misc/Hyperlinks.xlsx
@@ -509,15 +509,15 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink ref="A1" r:id="rId13"/>
-    <x:hyperlink ref="A2" r:id="rId14" tooltip="Click to go to Yahoo!"/>
+    <x:hyperlink ref="A1" r:id="rId6"/>
+    <x:hyperlink ref="A2" r:id="rId7" tooltip="Click to go to Yahoo!"/>
     <x:hyperlink ref="A3" location="Hyperlinks!Test.xlsx" display="Link to a file - same folder"/>
-    <x:hyperlink ref="A4" r:id="rId15"/>
-    <x:hyperlink ref="A5" r:id="rId16"/>
+    <x:hyperlink ref="A4" r:id="rId8"/>
+    <x:hyperlink ref="A5" r:id="rId9"/>
     <x:hyperlink ref="A6" location="Hyperlinks!B1" display="Link to an address in this worksheet"/>
     <x:hyperlink ref="A7" location="'Second Sheet'!A1" display="Link to an address in another worksheet"/>
     <x:hyperlink ref="A8" location="Hyperlinks!B1:C2" tooltip="SquareBox" display="Link to a range in this worksheet"/>
-    <x:hyperlink ref="A9" r:id="rId17"/>
+    <x:hyperlink ref="A9" r:id="rId10"/>
     <x:hyperlink ref="A11" location="Hyperlinks!B1:C2" display="Odd looking link"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>

</xml_diff>